<commit_message>
UI redesign and phase 2 milestone 8 , 9 implementation
</commit_message>
<xml_diff>
--- a/docs/MeetCopilot-Phase2-Testing-Checklist.xlsx
+++ b/docs/MeetCopilot-Phase2-Testing-Checklist.xlsx
@@ -101,7 +101,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -123,11 +123,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,6 +202,8 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -640,7 +686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1007,9 +1053,39 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="58" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Release feed for auto-update and hosts the signed installer the website links to.</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Repo (Devkolsawala/AI-Meeting-Assistant) + a personal access token with 'repo' scope to publish releases.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>GH_TOKEN</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Required (M8)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="F2:F13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Blocked,N/A,Done"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,N/A,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1023,7 +1099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1333,9 +1409,54 @@
       </c>
       <c r="E14" s="4" t="inlineStr"/>
     </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Create a GitHub token for releases</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Personal access token with 'repo' scope -&gt; GH_TOKEN, so electron-builder can upload release assets.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Publish signed release + set download URL</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Local build + Vercel</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Run pnpm --filter @meetcopilot/desktop release (signing env + GH_TOKEN set); then set INSTALLER_DOWNLOAD_URL to https://github.com/Devkolsawala/AI-Meeting-Assistant/releases/latest/download/MeetCopilot-Setup.exe and redeploy.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="E2:E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E15:E16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1349,7 +1470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1398,6 +1519,11 @@
           <t>M1 — Usage metering (apps/api)</t>
         </is>
       </c>
+      <c r="B2" s="12" t="n"/>
+      <c r="C2" s="12" t="n"/>
+      <c r="D2" s="12" t="n"/>
+      <c r="E2" s="12" t="n"/>
+      <c r="F2" s="13" t="n"/>
     </row>
     <row r="3" ht="50" customHeight="1">
       <c r="A3" s="8" t="n">
@@ -1471,6 +1597,11 @@
           <t>M2 — Plan gating + free cap (server-side)</t>
         </is>
       </c>
+      <c r="B6" s="12" t="n"/>
+      <c r="C6" s="12" t="n"/>
+      <c r="D6" s="12" t="n"/>
+      <c r="E6" s="12" t="n"/>
+      <c r="F6" s="13" t="n"/>
     </row>
     <row r="7" ht="50" customHeight="1">
       <c r="A7" s="8" t="n">
@@ -1588,6 +1719,11 @@
           <t>M3 — Deploy API to AWS App Runner</t>
         </is>
       </c>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="13" t="n"/>
     </row>
     <row r="13" ht="50" customHeight="1">
       <c r="A13" s="8" t="n">
@@ -1705,6 +1841,11 @@
           <t>M4 — Payments via Razorpay</t>
         </is>
       </c>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="13" t="n"/>
     </row>
     <row r="19" ht="50" customHeight="1">
       <c r="A19" s="8" t="n">
@@ -1822,6 +1963,11 @@
           <t>M5 — Account dashboard (apps/web /account)</t>
         </is>
       </c>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="13" t="n"/>
     </row>
     <row r="25" ht="50" customHeight="1">
       <c r="A25" s="8" t="n">
@@ -1939,6 +2085,11 @@
           <t>M6 — Observability (all 3 apps)</t>
         </is>
       </c>
+      <c r="B30" s="12" t="n"/>
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="13" t="n"/>
     </row>
     <row r="31" ht="50" customHeight="1">
       <c r="A31" s="8" t="n">
@@ -2034,6 +2185,11 @@
           <t>M7 — Desktop packaging + Windows code signing</t>
         </is>
       </c>
+      <c r="B35" s="12" t="n"/>
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="13" t="n"/>
     </row>
     <row r="36" ht="50" customHeight="1">
       <c r="A36" s="8" t="n">
@@ -2123,18 +2279,309 @@
       <c r="E39" s="4" t="inlineStr"/>
       <c r="F39" s="4" t="inlineStr"/>
     </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>M8 — Auto-update + website installer</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="n"/>
+      <c r="C40" s="12" t="n"/>
+      <c r="D40" s="12" t="n"/>
+      <c r="E40" s="12" t="n"/>
+      <c r="F40" s="13" t="n"/>
+    </row>
+    <row r="41" ht="50" customHeight="1">
+      <c r="A41" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Installer + update files build</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Set the cache env; run pnpm --filter @meetcopilot/desktop package.</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>release/ contains MeetCopilot-Setup.exe, MeetCopilot-Setup.exe.blockmap, and latest.yml.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr"/>
+    </row>
+    <row r="42" ht="50" customHeight="1">
+      <c r="A42" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Publish a GitHub release</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Set signing env + GH_TOKEN; run pnpm --filter @meetcopilot/desktop release.</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>A GitHub release is created with the installer + latest.yml + blockmap uploaded.</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="50" customHeight="1">
+      <c r="A43" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Website serves the signed installer</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Set INSTALLER_DOWNLOAD_URL to .../releases/latest/download/MeetCopilot-Setup.exe in Vercel; redeploy; click Download for Windows.</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Browser downloads the signed MeetCopilot-Setup.exe; it installs with no Unknown Publisher warning.</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="50" customHeight="1">
+      <c r="A44" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>App auto-updates itself</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Install release N, then publish release N+1 (bumped version). Relaunch the installed app.</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>diagnostics.log shows AUTO_UPDATE available N+1 -&gt; downloaded; after quit + reopen the app runs N+1.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45" ht="50" customHeight="1">
+      <c r="A45" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Dev run skips update</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Run unpackaged: pnpm --filter @meetcopilot/desktop start.</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Log shows 'AUTO_UPDATE skipped (app not packaged)'; no auto-update errors.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>M9 — First-run onboarding (apps/desktop)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="50" customHeight="1">
+      <c r="A47" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>Wizard shows on first run</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Fresh profile (delete %APPDATA%\MeetCopilot\onboarding.json), launch the app.</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>The 'Set up MeetCopilot' wizard covers the overlay with Microphone and System audio steps.</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48" ht="50" customHeight="1">
+      <c r="A48" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Microphone check passes</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Click 'Allow microphone' and accept any Windows prompt.</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Dot turns green, 'Microphone is ready.', button shows 'Microphone allowed'.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49" ht="50" customHeight="1">
+      <c r="A49" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>System audio check passes</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Click 'Test system audio' and allow screen capture.</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>Dot turns green, 'System audio is working.' (a loopback audio track was detected).</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50" ht="50" customHeight="1">
+      <c r="A50" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>Missing permission is detected</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Deny the microphone (or block it in Windows privacy settings) and click 'Allow microphone'.</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>Dot turns red with a clear message pointing to Troubleshooting; the app does not crash.</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51" ht="50" customHeight="1">
+      <c r="A51" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>Troubleshooting link works</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Click 'Troubleshooting'.</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>The browser opens &lt;WEB_URL&gt;/help/windows-audio with the Windows audio steps.</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52" ht="50" customHeight="1">
+      <c r="A52" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>Finish persists</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Click 'Finish setup', then fully quit and relaunch the app.</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>Wizard closes to the normal overlay; on relaunch it does NOT show again (onboarding.json -&gt; completed).</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53" ht="50" customHeight="1">
+      <c r="A53" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>New user sets up unattended</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>On a clean machine, install -&gt; launch -&gt; follow the wizard with no other guidance.</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Both audio sources end green and the user reaches a working overlay without external help.</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A46:F46"/>
     <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A40:F40"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A30:F30"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="3">
     <dataValidation sqref="E2:E39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Blocked,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E41:E45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Blocked,N/A"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E47:E53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>